<commit_message>
add date and report name generation to CC WSR
</commit_message>
<xml_diff>
--- a/services/ami/ami/ami_weekly_status_report/per_project/Complete_Chaos/Complete_Chaos_wsr_template.xlsx
+++ b/services/ami/ami/ami_weekly_status_report/per_project/Complete_Chaos/Complete_Chaos_wsr_template.xlsx
@@ -95,10 +95,10 @@
     <t xml:space="preserve">RVX</t>
   </si>
   <si>
-    <t xml:space="preserve">RVX_WeeklyReport_{date}_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{date}</t>
+    <t xml:space="preserve">{_report_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{_date}</t>
   </si>
   <si>
     <t xml:space="preserve">Shot</t>
@@ -122,7 +122,7 @@
     <t xml:space="preserve">{sg_next_delivery}</t>
   </si>
   <si>
-    <t xml:space="preserve">{sg__}%</t>
+    <t xml:space="preserve">{sg__}</t>
   </si>
   <si>
     <t xml:space="preserve">{sg_anim_blocking_date}</t>
@@ -274,7 +274,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U1048576"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.33"/>
@@ -519,9 +519,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="16" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.33"/>
   </cols>
   <sheetData>

</xml_diff>